<commit_message>
Resample code in ASM
</commit_message>
<xml_diff>
--- a/GBADoomMemory.xlsx
+++ b/GBADoomMemory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\GBADoom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BB6963-54E6-44D3-92CA-F06094FEEEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DC79FF-FA70-4B67-86A3-BA23E9C9797B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2850" yWindow="2850" windowWidth="25950" windowHeight="12630" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" r:id="rId1"/>
@@ -30501,6 +30501,162 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{00000000-0003-0000-0600-000000000000}">
+          <x14:colorSeries rgb="FF376092"/>
+          <x14:colorNegative rgb="FFD00000"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers rgb="FFD00000"/>
+          <x14:colorFirst rgb="FFD00000"/>
+          <x14:colorLast rgb="FFD00000"/>
+          <x14:colorHigh rgb="FFD00000"/>
+          <x14:colorLow rgb="FFD00000"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G2:G2</xm:f>
+              <xm:sqref>H2</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G3:G3</xm:f>
+              <xm:sqref>H3</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G4:G4</xm:f>
+              <xm:sqref>H4</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G5:G5</xm:f>
+              <xm:sqref>H5</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G6:G6</xm:f>
+              <xm:sqref>H6</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G7:G7</xm:f>
+              <xm:sqref>H7</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G8:G8</xm:f>
+              <xm:sqref>H8</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G9:G9</xm:f>
+              <xm:sqref>H9</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G10:G10</xm:f>
+              <xm:sqref>H10</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G11:G11</xm:f>
+              <xm:sqref>H11</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G12:G12</xm:f>
+              <xm:sqref>H12</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G13:G13</xm:f>
+              <xm:sqref>H13</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G14:G14</xm:f>
+              <xm:sqref>H14</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G15:G15</xm:f>
+              <xm:sqref>H15</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G16:G16</xm:f>
+              <xm:sqref>H16</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G17:G17</xm:f>
+              <xm:sqref>H17</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G18:G18</xm:f>
+              <xm:sqref>H18</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G19:G19</xm:f>
+              <xm:sqref>H19</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G20:G20</xm:f>
+              <xm:sqref>H20</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G21:G21</xm:f>
+              <xm:sqref>H21</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G22:G22</xm:f>
+              <xm:sqref>H22</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G23:G23</xm:f>
+              <xm:sqref>H23</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G24:G24</xm:f>
+              <xm:sqref>H24</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G25:G25</xm:f>
+              <xm:sqref>H25</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G26:G26</xm:f>
+              <xm:sqref>H26</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G27:G27</xm:f>
+              <xm:sqref>H27</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G28:G28</xm:f>
+              <xm:sqref>H28</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G29:G29</xm:f>
+              <xm:sqref>H29</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G30:G30</xm:f>
+              <xm:sqref>H30</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G31:G31</xm:f>
+              <xm:sqref>H31</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G32:G32</xm:f>
+              <xm:sqref>H32</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G33:G33</xm:f>
+              <xm:sqref>H33</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G34:G34</xm:f>
+              <xm:sqref>H34</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G35:G35</xm:f>
+              <xm:sqref>H35</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G36:G36</xm:f>
+              <xm:sqref>H36</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Doom Levels'!G37:G37</xm:f>
+              <xm:sqref>H37</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
         <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{00000000-0003-0000-0600-000001000000}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
@@ -30657,162 +30813,6 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{00000000-0003-0000-0600-000000000000}">
-          <x14:colorSeries rgb="FF376092"/>
-          <x14:colorNegative rgb="FFD00000"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers rgb="FFD00000"/>
-          <x14:colorFirst rgb="FFD00000"/>
-          <x14:colorLast rgb="FFD00000"/>
-          <x14:colorHigh rgb="FFD00000"/>
-          <x14:colorLow rgb="FFD00000"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G2:G2</xm:f>
-              <xm:sqref>H2</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G3:G3</xm:f>
-              <xm:sqref>H3</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G4:G4</xm:f>
-              <xm:sqref>H4</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G5:G5</xm:f>
-              <xm:sqref>H5</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G6:G6</xm:f>
-              <xm:sqref>H6</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G7:G7</xm:f>
-              <xm:sqref>H7</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G8:G8</xm:f>
-              <xm:sqref>H8</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G9:G9</xm:f>
-              <xm:sqref>H9</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G10:G10</xm:f>
-              <xm:sqref>H10</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G11:G11</xm:f>
-              <xm:sqref>H11</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G12:G12</xm:f>
-              <xm:sqref>H12</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G13:G13</xm:f>
-              <xm:sqref>H13</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G14:G14</xm:f>
-              <xm:sqref>H14</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G15:G15</xm:f>
-              <xm:sqref>H15</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G16:G16</xm:f>
-              <xm:sqref>H16</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G17:G17</xm:f>
-              <xm:sqref>H17</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G18:G18</xm:f>
-              <xm:sqref>H18</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G19:G19</xm:f>
-              <xm:sqref>H19</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G20:G20</xm:f>
-              <xm:sqref>H20</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G21:G21</xm:f>
-              <xm:sqref>H21</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G22:G22</xm:f>
-              <xm:sqref>H22</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G23:G23</xm:f>
-              <xm:sqref>H23</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G24:G24</xm:f>
-              <xm:sqref>H24</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G25:G25</xm:f>
-              <xm:sqref>H25</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G26:G26</xm:f>
-              <xm:sqref>H26</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G27:G27</xm:f>
-              <xm:sqref>H27</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G28:G28</xm:f>
-              <xm:sqref>H28</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G29:G29</xm:f>
-              <xm:sqref>H29</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G30:G30</xm:f>
-              <xm:sqref>H30</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G31:G31</xm:f>
-              <xm:sqref>H31</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G32:G32</xm:f>
-              <xm:sqref>H32</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G33:G33</xm:f>
-              <xm:sqref>H33</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G34:G34</xm:f>
-              <xm:sqref>H34</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G35:G35</xm:f>
-              <xm:sqref>H35</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G36:G36</xm:f>
-              <xm:sqref>H36</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Doom Levels'!G37:G37</xm:f>
-              <xm:sqref>H37</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
       </x14:sparklineGroups>
     </ext>
   </extLst>
@@ -32812,7 +32812,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{D21CAF72-2AF7-4E10-80D4-49E1123EB21E}">
+        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{00000000-0003-0000-0700-000002000000}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -32823,8 +32823,8 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Doom2 Levels'!L2:L2</xm:f>
-              <xm:sqref>M2</xm:sqref>
+              <xm:f>'Doom2 Levels'!G2:G2</xm:f>
+              <xm:sqref>H2</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
@@ -32844,7 +32844,7 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{00000000-0003-0000-0700-000002000000}">
+        <x14:sparklineGroup displayEmptyCellsAs="span" xr2:uid="{D21CAF72-2AF7-4E10-80D4-49E1123EB21E}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -32855,8 +32855,8 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Doom2 Levels'!G2:G2</xm:f>
-              <xm:sqref>H2</xm:sqref>
+              <xm:f>'Doom2 Levels'!L2:L2</xm:f>
+              <xm:sqref>M2</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
@@ -32868,13 +32868,13 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E70020B-64A4-492D-9830-6A4BD6B3C292}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -32894,7 +32894,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -32916,8 +32916,15 @@
       <c r="F2" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2">
+        <v>135868</v>
+      </c>
+      <c r="H2">
+        <f>B2-G2</f>
+        <v>46916</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -32939,8 +32946,15 @@
       <c r="F3" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3">
+        <v>152464</v>
+      </c>
+      <c r="H3">
+        <f>B3-G3</f>
+        <v>31384</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -32962,8 +32976,15 @@
       <c r="F4" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4">
+        <v>134404</v>
+      </c>
+      <c r="H4">
+        <f>B4-G4</f>
+        <v>17352</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -32985,8 +33006,15 @@
       <c r="F5" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5">
+        <v>209240</v>
+      </c>
+      <c r="H5">
+        <f>B5-G5</f>
+        <v>96552</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>89</v>
       </c>
@@ -33008,8 +33036,15 @@
       <c r="F6" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6">
+        <v>210800</v>
+      </c>
+      <c r="H6">
+        <f>B6-G6</f>
+        <v>25620</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -33031,8 +33066,15 @@
       <c r="F7" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7">
+        <v>221372</v>
+      </c>
+      <c r="H7">
+        <f>B7-G7</f>
+        <v>131088</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>91</v>
       </c>
@@ -33054,8 +33096,15 @@
       <c r="F8" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8">
+        <v>247984</v>
+      </c>
+      <c r="H8">
+        <f>B8-G8</f>
+        <v>134864</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>92</v>
       </c>
@@ -33078,7 +33127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>93</v>
       </c>

</xml_diff>